<commit_message>
incluído texto de falta de itens
</commit_message>
<xml_diff>
--- a/SIMULADOR_NIVEA_2026.xlsx
+++ b/SIMULADOR_NIVEA_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aliancanet-my.sharepoint.com/personal/isabelarodrigues_aliancanet_onmicrosoft_com/Documents/Cursos/ASIMOV/Projetos pessoais/nivea/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1539A53A-7232-498C-8E55-6F9FE1218DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{1539A53A-7232-498C-8E55-6F9FE1218DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D9998AB-1FA7-4D97-B19F-6C032179053B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -140,9 +140,6 @@
     <t>DES.NIVEA AERO FEM INV BLC WHT CLR 200ML</t>
   </si>
   <si>
-    <t>DES.NIVEA AERO FEM INV BLC WHT FRESH 150ML</t>
-  </si>
-  <si>
     <t>DES.NIVEA AERO FEM PEARL BEAUTY 200ML</t>
   </si>
   <si>
@@ -152,9 +149,6 @@
     <t>DES.NIVEA AERO FEM PROTECARE 200ML</t>
   </si>
   <si>
-    <t>DES.NIVEA AERO FEM PROTECARE 90GR</t>
-  </si>
-  <si>
     <t>DES.NIVEA AERO FEM SENS PURE S/PERF150ML</t>
   </si>
   <si>
@@ -212,12 +206,6 @@
     <t>DES.NIVEA ROLLON FEM PEARL BEAUTY 50ML</t>
   </si>
   <si>
-    <t>DES.NIVEA ROLLON FEM PROTECARE 2X50ML OF</t>
-  </si>
-  <si>
-    <t>DES.NIVEA ROLLON FEM PROTECARE 50ML</t>
-  </si>
-  <si>
     <t>DES.NIVEA ROLLON FEM SENS PURE S/P 50ML</t>
   </si>
   <si>
@@ -335,9 +323,6 @@
     <t>PROT.LABIAL NIVEA SUN FPS30 4,8GR</t>
   </si>
   <si>
-    <t>PROT.SOLAR NIVEA FACIAL OLEOS.FPS50 50GR</t>
-  </si>
-  <si>
     <t>PROT.SOLAR NIVEA FACIAL Q10 FPS30 40GR</t>
   </si>
   <si>
@@ -380,15 +365,6 @@
     <t>PROT.SOLAR NIVEA LOCAO FPS70 200ML</t>
   </si>
   <si>
-    <t>PROT.SOLAR NIVEA PEB FP30 200M+FP30 100M</t>
-  </si>
-  <si>
-    <t>PROT.SOLAR NIVEA PEB FPS30 125ML</t>
-  </si>
-  <si>
-    <t>PROT.SOLAR NIVEA PEB FPS30 200ML</t>
-  </si>
-  <si>
     <t>SAB.GEL NIVEA ACNE CONTROL 150G</t>
   </si>
   <si>
@@ -422,9 +398,6 @@
     <t>SAB.LIQ NIVEA ESFOL MASSAG CORP 200ML</t>
   </si>
   <si>
-    <t>SAB.LIQ NIVEA FRANGIPAN E OIL 250ML</t>
-  </si>
-  <si>
     <t>SAB.LIQ NIVEA INTIMO FRESH 250ML</t>
   </si>
   <si>
@@ -437,9 +410,6 @@
     <t>SAB.LIQ NIVEA NATURAL OIL 200ML</t>
   </si>
   <si>
-    <t>SAB.LIQ NIVEA WATER LILY E OIL 250ML</t>
-  </si>
-  <si>
     <t>SAB.NIVEA ANTIBAC 3 EM 1 12X85GR</t>
   </si>
   <si>
@@ -491,12 +461,6 @@
     <t>SAB.NIVEA HIDRAT TOQUE BAUNILHA 12X85GR</t>
   </si>
   <si>
-    <t>SAB. NIVEA VEG MANT DE CACAU &amp; JASMIN 12X80G</t>
-  </si>
-  <si>
-    <t>SAB. NIVEA VEG MANT DE KARITÉ &amp; LIMA 12X80G</t>
-  </si>
-  <si>
     <t>DES.NIVEA BARRA CLIN.FEM DERMA PROT.54GR</t>
   </si>
   <si>
@@ -506,15 +470,6 @@
     <t>DES.NIVEA AERO CLIN.MASC DERMA DEF.200ML</t>
   </si>
   <si>
-    <t>DES.NIVEA AERO CLIN.FEM DERMA DEFE.150ML</t>
-  </si>
-  <si>
-    <t>DES.NIVEA AERO CLIN.FEM DERMA REST.150ML</t>
-  </si>
-  <si>
-    <t>DES.NIVEA AERO CLIN.FEM DERMA UNIF.150ML</t>
-  </si>
-  <si>
     <t>DES.NIVEA AERO CLIN.FEM DERMA DEFE.200ML</t>
   </si>
   <si>
@@ -527,9 +482,6 @@
     <t>DES.NIVEA ROLLON FEM DERMA UNIF.50ML</t>
   </si>
   <si>
-    <t>DES.NIVEA AERO CLIN.MASC DERMA DEF.150ML</t>
-  </si>
-  <si>
     <t>SAB. NIVEA MAN KAR E L. DA PERSIA 6X80G</t>
   </si>
   <si>
@@ -554,12 +506,6 @@
     <t>TONICO NIVEA AQUA ROSE 200ML</t>
   </si>
   <si>
-    <t>SAB ABACATE E CAMOMILA 12X80G</t>
-  </si>
-  <si>
-    <t>SAB JOJOBA E FRAMBOESA 12X80G</t>
-  </si>
-  <si>
     <t>Categoria</t>
   </si>
   <si>
@@ -668,9 +614,6 @@
     <t>Valor Negociado REDE</t>
   </si>
   <si>
-    <t>DES.NIVEA ROLLON  MASC ORIG PROTECT 50ML</t>
-  </si>
-  <si>
     <t>CÓDIGO BIZ</t>
   </si>
   <si>
@@ -684,6 +627,63 @@
   </si>
   <si>
     <t>KIT.NIVEA PROT.SOLAR FPS70+CREME ANTISSI</t>
+  </si>
+  <si>
+    <t>DES.NIVEA AERO CONT.FEM DERMA DEFE.150ML</t>
+  </si>
+  <si>
+    <t>DES.NIVEA AERO CONT.FEM DERMA REST.150ML</t>
+  </si>
+  <si>
+    <t>DES.NIVEA AERO CONT.FEM DERMA UNIF.150ML</t>
+  </si>
+  <si>
+    <t>DES.NIVEA AERO CONT.MASC DERMA DEF.150ML</t>
+  </si>
+  <si>
+    <t>DES.NIVEA AERO FEM INV BL WH FRESH 150ML</t>
+  </si>
+  <si>
+    <t>DES.NIVEA AERO FEM PROT&amp;CARE 90GR</t>
+  </si>
+  <si>
+    <t>DES.NIVEA ROLLON MASC ORIG PROTECT 50ML</t>
+  </si>
+  <si>
+    <t>DES.NIVEA ROLLON FEM PROT&amp;CARE 2X50ML OF</t>
+  </si>
+  <si>
+    <t>DES.NIVEA ROLLON FEM PROT&amp;CARE 50ML</t>
+  </si>
+  <si>
+    <t>PROT.SOLAR NIVEA FAC.EF.MATTE FPS60 50GR</t>
+  </si>
+  <si>
+    <t>PROT.SOLAR NIVEA P&amp;B FP30 200M+FP30 100M</t>
+  </si>
+  <si>
+    <t>PROT.SOLAR NIVEA P&amp;B FPS30 125ML</t>
+  </si>
+  <si>
+    <t>PROT.SOLAR NIVEA P&amp;B FPS30 200ML</t>
+  </si>
+  <si>
+    <t>SAB. NIVEA OLEO ABACATE E CAMOMIL 12X80G</t>
+  </si>
+  <si>
+    <t>SAB. NIVEA OLEO JOJOBA E FRAMBOES 12X80G</t>
+  </si>
+  <si>
+    <t>SAB. NIVEA MANT CACAU E JASMIM 12X80G</t>
+  </si>
+  <si>
+    <t>SAB. NIVEA MAN KARITE E L.PERSIA 12X80G</t>
+  </si>
+  <si>
+    <t>SAB.LIQ NIVEA FRANGIPAN &amp; OIL 250ML</t>
+  </si>
+  <si>
+    <t>SAB.LIQ NIVEA WATER LILY &amp; OIL 250ML</t>
   </si>
 </sst>
 </file>
@@ -1740,10 +1740,10 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.6">
       <c r="A1" s="3" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -1755,12 +1755,12 @@
         <v>3</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>209</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="B2" s="1">
         <v>703209</v>
@@ -1776,7 +1776,7 @@
     </row>
     <row r="3" spans="1:6" ht="14.25" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="B3" s="1">
         <v>703217</v>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="4" spans="1:6" ht="14.25" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="B4" s="1">
         <v>701896</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="5" spans="1:6" ht="14.25" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="B5" s="1">
         <v>702168</v>
@@ -1828,7 +1828,7 @@
     </row>
     <row r="6" spans="1:6" ht="14.25" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="B6" s="1">
         <v>700109</v>
@@ -1840,13 +1840,13 @@
         <v>9</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:6" ht="14.25" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="B7" s="1">
         <v>700117</v>
@@ -1862,7 +1862,7 @@
     </row>
     <row r="8" spans="1:6" ht="14.25" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B8" s="1">
         <v>702584</v>
@@ -1874,13 +1874,13 @@
         <v>11</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" ht="14.25" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B9" s="1">
         <v>703465</v>
@@ -1896,7 +1896,7 @@
     </row>
     <row r="10" spans="1:6" ht="14.25" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B10" s="1">
         <v>702953</v>
@@ -1912,7 +1912,7 @@
     </row>
     <row r="11" spans="1:6" ht="14.25" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B11" s="1">
         <v>702753</v>
@@ -1930,7 +1930,7 @@
     </row>
     <row r="12" spans="1:6" ht="14.25" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B12" s="1">
         <v>702576</v>
@@ -1948,7 +1948,7 @@
     </row>
     <row r="13" spans="1:6" ht="14.25" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B13" s="1">
         <v>212964</v>
@@ -1966,7 +1966,7 @@
     </row>
     <row r="14" spans="1:6" ht="14.25" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B14" s="1">
         <v>703441</v>
@@ -1982,7 +1982,7 @@
     </row>
     <row r="15" spans="1:6" ht="14.25" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B15" s="1">
         <v>703449</v>
@@ -1998,7 +1998,7 @@
     </row>
     <row r="16" spans="1:6" ht="14.25" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B16" s="1">
         <v>700213</v>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="17" spans="1:6" ht="14.25" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="B17" s="1">
         <v>703185</v>
@@ -2030,7 +2030,7 @@
     </row>
     <row r="18" spans="1:6" ht="14.25" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="B18" s="1">
         <v>703193</v>
@@ -2046,7 +2046,7 @@
     </row>
     <row r="19" spans="1:6" ht="14.25" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="B19" s="1">
         <v>703177</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="20" spans="1:6" ht="14.25" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="B20" s="1">
         <v>700125</v>
@@ -2078,7 +2078,7 @@
     </row>
     <row r="21" spans="1:6" ht="14.25" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="B21" s="1">
         <v>702112</v>
@@ -2094,135 +2094,135 @@
     </row>
     <row r="22" spans="1:6" ht="14.25" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B22" s="1">
-        <v>703865</v>
+        <v>703921</v>
       </c>
       <c r="C22" s="2">
-        <v>4006000178851</v>
+        <v>4006000178868</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="7"/>
     </row>
     <row r="23" spans="1:6" ht="14.25" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B23" s="1">
-        <v>703921</v>
+        <v>703353</v>
       </c>
       <c r="C23" s="2">
-        <v>4006000178868</v>
+        <v>4005900950925</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>159</v>
+        <v>25</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="7"/>
     </row>
     <row r="24" spans="1:6" ht="14.25" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B24" s="1">
-        <v>703353</v>
+        <v>703361</v>
       </c>
       <c r="C24" s="2">
-        <v>4005900950925</v>
+        <v>4005900950918</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="7"/>
     </row>
     <row r="25" spans="1:6" ht="14.25" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B25" s="1">
-        <v>703889</v>
+        <v>703849</v>
       </c>
       <c r="C25" s="2">
-        <v>4006000178899</v>
+        <v>4006000178912</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="7"/>
     </row>
     <row r="26" spans="1:6" ht="14.25" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B26" s="1">
-        <v>703905</v>
+        <v>703865</v>
       </c>
       <c r="C26" s="2">
-        <v>4006000178882</v>
+        <v>4006000178851</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>158</v>
+        <v>197</v>
       </c>
       <c r="E26" s="5"/>
       <c r="F26" s="7"/>
     </row>
     <row r="27" spans="1:6" ht="14.25" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="B27" s="1">
-        <v>703361</v>
+        <v>703889</v>
       </c>
       <c r="C27" s="2">
-        <v>4005900950918</v>
+        <v>4006000178899</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>26</v>
+        <v>198</v>
       </c>
       <c r="E27" s="5"/>
       <c r="F27" s="7"/>
     </row>
     <row r="28" spans="1:6" ht="14.25" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>183</v>
+        <v>164</v>
       </c>
       <c r="B28" s="1">
-        <v>703841</v>
+        <v>703905</v>
       </c>
       <c r="C28" s="2">
-        <v>4006000178905</v>
+        <v>4006000178882</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>163</v>
+        <v>199</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="7"/>
     </row>
     <row r="29" spans="1:6" ht="14.25" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
       <c r="B29" s="1">
-        <v>703849</v>
+        <v>703841</v>
       </c>
       <c r="C29" s="2">
-        <v>4006000178912</v>
+        <v>4006000178905</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="7"/>
     </row>
     <row r="30" spans="1:6" ht="14.25" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B30" s="1">
         <v>703201</v>
@@ -2240,7 +2240,7 @@
     </row>
     <row r="31" spans="1:6" ht="14.25" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B31" s="1">
         <v>703401</v>
@@ -2256,7 +2256,7 @@
     </row>
     <row r="32" spans="1:6" ht="14.25" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B32" s="1">
         <v>700253</v>
@@ -2274,7 +2274,7 @@
     </row>
     <row r="33" spans="1:6" ht="14.25" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B33" s="1">
         <v>700237</v>
@@ -2290,7 +2290,7 @@
     </row>
     <row r="34" spans="1:6" ht="14.25" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B34" s="1">
         <v>703641</v>
@@ -2306,57 +2306,57 @@
     </row>
     <row r="35" spans="1:6" ht="14.25" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B35" s="1">
-        <v>700533</v>
+        <v>702368</v>
       </c>
       <c r="C35" s="2">
-        <v>4005900036667</v>
+        <v>4005900429643</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>175</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="E35" s="5"/>
       <c r="F35" s="7"/>
     </row>
     <row r="36" spans="1:6" ht="14.25" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="B36" s="1">
-        <v>703385</v>
+        <v>700533</v>
       </c>
       <c r="C36" s="2">
-        <v>4005900105073</v>
+        <v>4005900036667</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E36" s="5"/>
+        <v>32</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="F36" s="7"/>
     </row>
     <row r="37" spans="1:6" ht="14.25" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="B37" s="1">
-        <v>702368</v>
+        <v>703385</v>
       </c>
       <c r="C37" s="2">
-        <v>4005900429643</v>
+        <v>4005900105073</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E37" s="5"/>
       <c r="F37" s="7"/>
     </row>
     <row r="38" spans="1:6" ht="14.25" customHeight="1">
       <c r="A38" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B38" s="1">
         <v>703513</v>
@@ -2365,14 +2365,14 @@
         <v>4006000010328</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E38" s="5"/>
       <c r="F38" s="7"/>
     </row>
     <row r="39" spans="1:6" ht="14.25" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B39" s="1">
         <v>700397</v>
@@ -2381,7 +2381,7 @@
         <v>4005808837311</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E39" s="5" t="s">
         <v>5</v>
@@ -2390,41 +2390,41 @@
     </row>
     <row r="40" spans="1:6" ht="14.25" customHeight="1">
       <c r="A40" s="1" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="B40" s="1">
-        <v>703369</v>
+        <v>702056</v>
       </c>
       <c r="C40" s="2">
-        <v>4005900705143</v>
+        <v>4005900122186</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E40" s="5"/>
+        <v>202</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="F40" s="7"/>
     </row>
     <row r="41" spans="1:6" ht="14.25" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="B41" s="1">
-        <v>702056</v>
+        <v>703369</v>
       </c>
       <c r="C41" s="2">
-        <v>4005900122186</v>
+        <v>4005900705143</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>175</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="E41" s="5"/>
       <c r="F41" s="7"/>
     </row>
     <row r="42" spans="1:6" ht="14.25" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B42" s="1">
         <v>701053</v>
@@ -2433,14 +2433,14 @@
         <v>4005808662388</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E42" s="5"/>
       <c r="F42" s="7"/>
     </row>
     <row r="43" spans="1:6" ht="14.25" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B43" s="1">
         <v>702392</v>
@@ -2449,14 +2449,14 @@
         <v>4005900449559</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E43" s="5"/>
       <c r="F43" s="7"/>
     </row>
     <row r="44" spans="1:6" ht="14.25" customHeight="1">
       <c r="A44" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B44" s="1">
         <v>703377</v>
@@ -2465,14 +2465,14 @@
         <v>4005900105080</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="7"/>
     </row>
     <row r="45" spans="1:6" ht="14.25" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B45" s="1">
         <v>700549</v>
@@ -2481,16 +2481,16 @@
         <v>4005900036728</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F45" s="7"/>
     </row>
     <row r="46" spans="1:6" ht="14.25" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B46" s="1">
         <v>703009</v>
@@ -2499,14 +2499,14 @@
         <v>4005900707543</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="7"/>
     </row>
     <row r="47" spans="1:6" ht="14.25" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B47" s="1">
         <v>702993</v>
@@ -2515,7 +2515,7 @@
         <v>4005900707536</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>5</v>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="48" spans="1:6" ht="14.25" customHeight="1">
       <c r="A48" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B48" s="1">
         <v>703761</v>
@@ -2533,14 +2533,14 @@
         <v>4006000104256</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="7"/>
     </row>
     <row r="49" spans="1:6" ht="14.25" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B49" s="1">
         <v>703745</v>
@@ -2549,14 +2549,14 @@
         <v>4006000104164</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="7"/>
     </row>
     <row r="50" spans="1:6" ht="14.25" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B50" s="1">
         <v>703393</v>
@@ -2565,14 +2565,14 @@
         <v>4005900633309</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="7"/>
     </row>
     <row r="51" spans="1:6" ht="14.25" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B51" s="1">
         <v>700245</v>
@@ -2581,16 +2581,16 @@
         <v>7791969016029</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F51" s="7"/>
     </row>
     <row r="52" spans="1:6" ht="14.25" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B52" s="1">
         <v>703689</v>
@@ -2599,14 +2599,14 @@
         <v>4006000019338</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E52" s="5"/>
       <c r="F52" s="7"/>
     </row>
     <row r="53" spans="1:6" ht="14.25" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B53" s="1">
         <v>703521</v>
@@ -2615,14 +2615,14 @@
         <v>4006000010311</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E53" s="5"/>
       <c r="F53" s="7"/>
     </row>
     <row r="54" spans="1:6" ht="14.25" customHeight="1">
       <c r="A54" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B54" s="1">
         <v>702304</v>
@@ -2631,7 +2631,7 @@
         <v>4005900396938</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E54" s="5" t="s">
         <v>5</v>
@@ -2640,7 +2640,7 @@
     </row>
     <row r="55" spans="1:6" ht="14.25" customHeight="1">
       <c r="A55" s="1" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B55" s="1">
         <v>702136</v>
@@ -2649,14 +2649,14 @@
         <v>7791969029807</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E55" s="5"/>
       <c r="F55" s="7"/>
     </row>
     <row r="56" spans="1:6" ht="14.25" customHeight="1">
       <c r="A56" s="1" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="B56" s="1">
         <v>703929</v>
@@ -2665,14 +2665,14 @@
         <v>4006000045498</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="E56" s="5"/>
       <c r="F56" s="7"/>
     </row>
     <row r="57" spans="1:6" ht="14.25" customHeight="1">
       <c r="A57" s="1" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="B57" s="1">
         <v>703937</v>
@@ -2681,7 +2681,7 @@
         <v>4005805448299</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="7"/>
@@ -2691,13 +2691,13 @@
         <v>0</v>
       </c>
       <c r="B58" s="1">
-        <v>702312</v>
+        <v>703753</v>
       </c>
       <c r="C58" s="2">
-        <v>4005900398598</v>
+        <v>4006000104157</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>210</v>
+        <v>51</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="7"/>
@@ -2707,13 +2707,13 @@
         <v>0</v>
       </c>
       <c r="B59" s="1">
-        <v>703753</v>
+        <v>701784</v>
       </c>
       <c r="C59" s="2">
-        <v>4006000104157</v>
+        <v>4005900181046</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="7"/>
@@ -2723,15 +2723,17 @@
         <v>0</v>
       </c>
       <c r="B60" s="1">
-        <v>701784</v>
+        <v>700541</v>
       </c>
       <c r="C60" s="2">
-        <v>4005900181046</v>
+        <v>4005900036704</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E60" s="5"/>
+        <v>53</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="F60" s="7"/>
     </row>
     <row r="61" spans="1:6" ht="14.25" customHeight="1">
@@ -2739,17 +2741,15 @@
         <v>0</v>
       </c>
       <c r="B61" s="1">
-        <v>700541</v>
+        <v>703825</v>
       </c>
       <c r="C61" s="2">
-        <v>4005900036704</v>
+        <v>4006000181936</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>175</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="E61" s="5"/>
       <c r="F61" s="7"/>
     </row>
     <row r="62" spans="1:6" ht="14.25" customHeight="1">
@@ -2757,13 +2757,13 @@
         <v>0</v>
       </c>
       <c r="B62" s="1">
-        <v>703825</v>
+        <v>703817</v>
       </c>
       <c r="C62" s="2">
-        <v>4006000181936</v>
+        <v>4006000181950</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="7"/>
@@ -2773,13 +2773,13 @@
         <v>0</v>
       </c>
       <c r="B63" s="1">
-        <v>703817</v>
+        <v>703833</v>
       </c>
       <c r="C63" s="2">
-        <v>4006000181950</v>
+        <v>4006000181943</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="7"/>
@@ -2789,15 +2789,17 @@
         <v>0</v>
       </c>
       <c r="B64" s="1">
-        <v>703833</v>
+        <v>700269</v>
       </c>
       <c r="C64" s="2">
-        <v>4006000181943</v>
+        <v>4005808257584</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="E64" s="5"/>
+        <v>54</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>5</v>
+      </c>
       <c r="F64" s="7"/>
     </row>
     <row r="65" spans="1:6" ht="14.25" customHeight="1">
@@ -2805,17 +2807,15 @@
         <v>0</v>
       </c>
       <c r="B65" s="1">
-        <v>700269</v>
+        <v>700405</v>
       </c>
       <c r="C65" s="2">
-        <v>4005808257584</v>
+        <v>4005808257669</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>5</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="E65" s="5"/>
       <c r="F65" s="7"/>
     </row>
     <row r="66" spans="1:6" ht="14.25" customHeight="1">
@@ -2823,13 +2823,13 @@
         <v>0</v>
       </c>
       <c r="B66" s="1">
-        <v>700405</v>
+        <v>702096</v>
       </c>
       <c r="C66" s="2">
-        <v>4005808257669</v>
+        <v>4005900359124</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>57</v>
+        <v>204</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="7"/>
@@ -2839,13 +2839,13 @@
         <v>0</v>
       </c>
       <c r="B67" s="1">
-        <v>702096</v>
+        <v>701808</v>
       </c>
       <c r="C67" s="2">
-        <v>4005900359124</v>
+        <v>4005900130785</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>58</v>
+        <v>205</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="7"/>
@@ -2855,13 +2855,13 @@
         <v>0</v>
       </c>
       <c r="B68" s="1">
-        <v>701808</v>
+        <v>701069</v>
       </c>
       <c r="C68" s="2">
-        <v>4005900130785</v>
+        <v>4005808663927</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="7"/>
@@ -2871,13 +2871,13 @@
         <v>0</v>
       </c>
       <c r="B69" s="1">
-        <v>701069</v>
+        <v>701792</v>
       </c>
       <c r="C69" s="2">
-        <v>4005808663927</v>
+        <v>4005900181039</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="7"/>
@@ -2887,15 +2887,17 @@
         <v>0</v>
       </c>
       <c r="B70" s="1">
-        <v>701792</v>
+        <v>700557</v>
       </c>
       <c r="C70" s="2">
-        <v>4005900181039</v>
+        <v>4005900036759</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E70" s="5"/>
+        <v>58</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="F70" s="7"/>
     </row>
     <row r="71" spans="1:6" ht="14.25" customHeight="1">
@@ -2903,16 +2905,16 @@
         <v>0</v>
       </c>
       <c r="B71" s="1">
-        <v>700557</v>
+        <v>700261</v>
       </c>
       <c r="C71" s="2">
-        <v>4005900036759</v>
+        <v>4005808257553</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>175</v>
+        <v>5</v>
       </c>
       <c r="F71" s="7"/>
     </row>
@@ -2921,22 +2923,20 @@
         <v>0</v>
       </c>
       <c r="B72" s="1">
-        <v>700261</v>
+        <v>702312</v>
       </c>
       <c r="C72" s="2">
-        <v>4005808257553</v>
+        <v>4005900398598</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E72" s="5" t="s">
-        <v>5</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="E72" s="5"/>
       <c r="F72" s="7"/>
     </row>
     <row r="73" spans="1:6" ht="14.25" customHeight="1">
       <c r="A73" s="1" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="B73" s="1">
         <v>703713</v>
@@ -2945,7 +2945,7 @@
         <v>4006000088112</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="7"/>
@@ -2961,14 +2961,14 @@
         <v>4006000085487</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E74" s="5"/>
       <c r="F74" s="7"/>
     </row>
     <row r="75" spans="1:6" ht="14.25" customHeight="1">
       <c r="A75" s="1" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="B75" s="1">
         <v>703481</v>
@@ -2977,14 +2977,14 @@
         <v>4005900940759</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E75" s="5"/>
       <c r="F75" s="7"/>
     </row>
     <row r="76" spans="1:6" ht="14.25" customHeight="1">
       <c r="A76" s="1" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B76" s="1">
         <v>703017</v>
@@ -2993,14 +2993,14 @@
         <v>4005900648327</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="7"/>
     </row>
     <row r="77" spans="1:6" ht="14.25" customHeight="1">
       <c r="A77" s="1" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B77" s="1">
         <v>702080</v>
@@ -3009,14 +3009,14 @@
         <v>4005808817009</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E77" s="5"/>
       <c r="F77" s="7"/>
     </row>
     <row r="78" spans="1:6" ht="14.25" customHeight="1">
       <c r="A78" s="1" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B78" s="1">
         <v>702144</v>
@@ -3025,7 +3025,7 @@
         <v>4005808817207</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E78" s="5" t="s">
         <v>5</v>
@@ -3034,7 +3034,7 @@
     </row>
     <row r="79" spans="1:6" ht="14.25" customHeight="1">
       <c r="A79" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B79" s="1">
         <v>703657</v>
@@ -3043,14 +3043,14 @@
         <v>4006000039800</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E79" s="5"/>
       <c r="F79" s="7"/>
     </row>
     <row r="80" spans="1:6" ht="14.25" customHeight="1">
       <c r="A80" s="1" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="B80" s="1">
         <v>703321</v>
@@ -3059,7 +3059,7 @@
         <v>4005900919632</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E80" s="5" t="s">
         <v>5</v>
@@ -3068,7 +3068,7 @@
     </row>
     <row r="81" spans="1:6" ht="14.25" customHeight="1">
       <c r="A81" s="1" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="B81" s="1">
         <v>703329</v>
@@ -3077,14 +3077,14 @@
         <v>4005900929365</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E81" s="5"/>
       <c r="F81" s="7"/>
     </row>
     <row r="82" spans="1:6" ht="14.25" customHeight="1">
       <c r="A82" s="1" t="s">
-        <v>191</v>
+        <v>173</v>
       </c>
       <c r="B82" s="1">
         <v>703313</v>
@@ -3093,14 +3093,14 @@
         <v>4005900919625</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E82" s="5"/>
       <c r="F82" s="7"/>
     </row>
     <row r="83" spans="1:6" ht="14.25" customHeight="1">
       <c r="A83" s="1" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="B83" s="1">
         <v>703497</v>
@@ -3109,14 +3109,14 @@
         <v>4005900945693</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="7"/>
     </row>
     <row r="84" spans="1:6" ht="14.25" customHeight="1">
       <c r="A84" s="1" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="B84" s="1">
         <v>702536</v>
@@ -3125,14 +3125,14 @@
         <v>4005900498205</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="7"/>
     </row>
     <row r="85" spans="1:6" ht="14.25" customHeight="1">
       <c r="A85" s="1" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="B85" s="1">
         <v>703561</v>
@@ -3141,14 +3141,14 @@
         <v>4005900549266</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="7"/>
     </row>
     <row r="86" spans="1:6" ht="14.25" customHeight="1">
       <c r="A86" s="1" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="B86" s="1">
         <v>700101</v>
@@ -3157,14 +3157,14 @@
         <v>4005808311286</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E86" s="5"/>
       <c r="F86" s="7"/>
     </row>
     <row r="87" spans="1:6" ht="14.25" customHeight="1">
       <c r="A87" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B87" s="1">
         <v>701984</v>
@@ -3173,14 +3173,14 @@
         <v>4005900116192</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E87" s="5"/>
       <c r="F87" s="7"/>
     </row>
     <row r="88" spans="1:6" ht="14.25" customHeight="1">
       <c r="A88" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B88" s="1">
         <v>700053</v>
@@ -3189,14 +3189,14 @@
         <v>4005808310999</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E88" s="5"/>
       <c r="F88" s="7"/>
     </row>
     <row r="89" spans="1:6" ht="14.25" customHeight="1">
       <c r="A89" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B89" s="1">
         <v>700013</v>
@@ -3205,16 +3205,16 @@
         <v>4005808309436</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F89" s="7"/>
     </row>
     <row r="90" spans="1:6" ht="14.25" customHeight="1">
       <c r="A90" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B90" s="1">
         <v>703337</v>
@@ -3223,14 +3223,14 @@
         <v>4005900441942</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E90" s="5"/>
       <c r="F90" s="7"/>
     </row>
     <row r="91" spans="1:6" ht="14.25" customHeight="1">
       <c r="A91" s="1" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="B91" s="1">
         <v>701912</v>
@@ -3239,7 +3239,7 @@
         <v>4005808315697</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>5</v>
@@ -3248,7 +3248,7 @@
     </row>
     <row r="92" spans="1:6" ht="14.25" customHeight="1">
       <c r="A92" s="1" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="B92" s="1">
         <v>701405</v>
@@ -3257,14 +3257,14 @@
         <v>4005808840625</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="7"/>
     </row>
     <row r="93" spans="1:6" ht="14.25" customHeight="1">
       <c r="A93" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B93" s="1">
         <v>703665</v>
@@ -3273,14 +3273,14 @@
         <v>4006000046686</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="E93" s="5"/>
       <c r="F93" s="7"/>
     </row>
     <row r="94" spans="1:6" ht="14.25" customHeight="1">
       <c r="A94" s="1" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B94" s="1">
         <v>700061</v>
@@ -3289,7 +3289,7 @@
         <v>4005808335435</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E94" s="5" t="s">
         <v>5</v>
@@ -3298,7 +3298,7 @@
     </row>
     <row r="95" spans="1:6" ht="14.25" customHeight="1">
       <c r="A95" s="1" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="B95" s="1">
         <v>701960</v>
@@ -3307,7 +3307,7 @@
         <v>4005900004956</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>5</v>
@@ -3316,7 +3316,7 @@
     </row>
     <row r="96" spans="1:6" ht="14.25" customHeight="1">
       <c r="A96" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B96" s="1">
         <v>703953</v>
@@ -3325,14 +3325,14 @@
         <v>4006000136776</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
       <c r="E96" s="5"/>
       <c r="F96" s="7"/>
     </row>
     <row r="97" spans="1:6" ht="14.25" customHeight="1">
       <c r="A97" s="1" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="B97" s="1">
         <v>703577</v>
@@ -3341,14 +3341,14 @@
         <v>4006000005430</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E97" s="5"/>
       <c r="F97" s="7"/>
     </row>
     <row r="98" spans="1:6" ht="14.25" customHeight="1">
       <c r="A98" s="1" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B98" s="1">
         <v>700901</v>
@@ -3357,14 +3357,14 @@
         <v>8715200813061</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="7"/>
     </row>
     <row r="99" spans="1:6" ht="14.25" customHeight="1">
       <c r="A99" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B99" s="1">
         <v>703697</v>
@@ -3373,14 +3373,14 @@
         <v>4005900991874</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E99" s="5"/>
       <c r="F99" s="7"/>
     </row>
     <row r="100" spans="1:6" ht="14.25" customHeight="1">
       <c r="A100" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B100" s="1">
         <v>702945</v>
@@ -3389,14 +3389,14 @@
         <v>4005900453259</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E100" s="5"/>
       <c r="F100" s="7"/>
     </row>
     <row r="101" spans="1:6" ht="14.25" customHeight="1">
       <c r="A101" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B101" s="1">
         <v>703881</v>
@@ -3405,14 +3405,14 @@
         <v>4006000159195</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="E101" s="5"/>
       <c r="F101" s="7"/>
     </row>
     <row r="102" spans="1:6" ht="14.25" customHeight="1">
       <c r="A102" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B102" s="1">
         <v>703649</v>
@@ -3421,14 +3421,14 @@
         <v>4005900663993</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E102" s="5"/>
       <c r="F102" s="7"/>
     </row>
     <row r="103" spans="1:6" ht="14.25" customHeight="1">
       <c r="A103" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B103" s="1">
         <v>703265</v>
@@ -3437,14 +3437,14 @@
         <v>4005900921567</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="7"/>
     </row>
     <row r="104" spans="1:6" ht="14.25" customHeight="1">
       <c r="A104" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B104" s="1">
         <v>703257</v>
@@ -3453,14 +3453,14 @@
         <v>4005900921598</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="7"/>
     </row>
     <row r="105" spans="1:6" ht="14.25" customHeight="1">
       <c r="A105" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B105" s="1">
         <v>703273</v>
@@ -3469,14 +3469,14 @@
         <v>4005900921574</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E105" s="5"/>
       <c r="F105" s="7"/>
     </row>
     <row r="106" spans="1:6" ht="14.25" customHeight="1">
       <c r="A106" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B106" s="1">
         <v>702176</v>
@@ -3485,14 +3485,14 @@
         <v>4005808369621</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E106" s="5"/>
       <c r="F106" s="7"/>
     </row>
     <row r="107" spans="1:6" ht="14.25" customHeight="1">
       <c r="A107" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B107" s="1">
         <v>702240</v>
@@ -3501,14 +3501,14 @@
         <v>4005808934980</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E107" s="5"/>
       <c r="F107" s="7"/>
     </row>
     <row r="108" spans="1:6" ht="14.25" customHeight="1">
       <c r="A108" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B108" s="1">
         <v>703857</v>
@@ -3517,14 +3517,14 @@
         <v>4006000159188</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="E108" s="5"/>
       <c r="F108" s="7"/>
     </row>
     <row r="109" spans="1:6" ht="14.25" customHeight="1">
       <c r="A109" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B109" s="1">
         <v>702016</v>
@@ -3533,7 +3533,7 @@
         <v>4005808850839</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>5</v>
@@ -3542,7 +3542,7 @@
     </row>
     <row r="110" spans="1:6" ht="14.25" customHeight="1">
       <c r="A110" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B110" s="1">
         <v>702008</v>
@@ -3551,7 +3551,7 @@
         <v>4005808850617</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>5</v>
@@ -3560,7 +3560,7 @@
     </row>
     <row r="111" spans="1:6" ht="14.25" customHeight="1">
       <c r="A111" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B111" s="1">
         <v>703873</v>
@@ -3569,14 +3569,14 @@
         <v>4006000159171</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="E111" s="5"/>
       <c r="F111" s="7"/>
     </row>
     <row r="112" spans="1:6" ht="14.25" customHeight="1">
       <c r="A112" s="1" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B112" s="1">
         <v>700141</v>
@@ -3585,14 +3585,14 @@
         <v>7890704851335</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E112" s="5"/>
       <c r="F112" s="7"/>
     </row>
     <row r="113" spans="1:6" ht="14.25" customHeight="1">
       <c r="A113" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B113" s="1">
         <v>703145</v>
@@ -3601,14 +3601,14 @@
         <v>4005900659712</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>99</v>
+        <v>206</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="7"/>
     </row>
     <row r="114" spans="1:6" ht="14.25" customHeight="1">
       <c r="A114" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B114" s="1">
         <v>703681</v>
@@ -3617,14 +3617,14 @@
         <v>4005900980380</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E114" s="5"/>
       <c r="F114" s="7"/>
     </row>
     <row r="115" spans="1:6" ht="14.25" customHeight="1">
       <c r="A115" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B115" s="1">
         <v>703169</v>
@@ -3633,14 +3633,14 @@
         <v>4005900646491</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E115" s="5"/>
       <c r="F115" s="7"/>
     </row>
     <row r="116" spans="1:6" ht="14.25" customHeight="1">
       <c r="A116" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B116" s="1">
         <v>703137</v>
@@ -3649,14 +3649,14 @@
         <v>4005900837677</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E116" s="5"/>
       <c r="F116" s="7"/>
     </row>
     <row r="117" spans="1:6" ht="14.25" customHeight="1">
       <c r="A117" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B117" s="1">
         <v>702528</v>
@@ -3665,14 +3665,14 @@
         <v>4005900980397</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E117" s="5"/>
       <c r="F117" s="7"/>
     </row>
     <row r="118" spans="1:6" ht="14.25" customHeight="1">
       <c r="A118" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B118" s="1">
         <v>700725</v>
@@ -3681,14 +3681,14 @@
         <v>4005808555321</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E118" s="5"/>
       <c r="F118" s="7"/>
     </row>
     <row r="119" spans="1:6" ht="14.25" customHeight="1">
       <c r="A119" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B119" s="1">
         <v>700733</v>
@@ -3697,7 +3697,7 @@
         <v>4005808555307</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>5</v>
@@ -3706,7 +3706,7 @@
     </row>
     <row r="120" spans="1:6" ht="14.25" customHeight="1">
       <c r="A120" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B120" s="1">
         <v>703409</v>
@@ -3715,14 +3715,14 @@
         <v>4005900695543</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E120" s="5"/>
       <c r="F120" s="7"/>
     </row>
     <row r="121" spans="1:6" ht="14.25" customHeight="1">
       <c r="A121" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B121" s="1">
         <v>700741</v>
@@ -3731,14 +3731,14 @@
         <v>4005808555352</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E121" s="5"/>
       <c r="F121" s="7"/>
     </row>
     <row r="122" spans="1:6" ht="14.25" customHeight="1">
       <c r="A122" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B122" s="1">
         <v>703417</v>
@@ -3747,14 +3747,14 @@
         <v>4005900695536</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E122" s="5"/>
       <c r="F122" s="7"/>
     </row>
     <row r="123" spans="1:6" ht="14.25" customHeight="1">
       <c r="A123" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B123" s="1">
         <v>700749</v>
@@ -3763,7 +3763,7 @@
         <v>4005808555345</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>5</v>
@@ -3772,7 +3772,7 @@
     </row>
     <row r="124" spans="1:6" ht="14.25" customHeight="1">
       <c r="A124" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B124" s="1">
         <v>703737</v>
@@ -3781,14 +3781,14 @@
         <v>4005900709752</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="7"/>
     </row>
     <row r="125" spans="1:6" ht="14.25" customHeight="1">
       <c r="A125" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B125" s="1">
         <v>701664</v>
@@ -3797,14 +3797,14 @@
         <v>4005808838899</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E125" s="5"/>
       <c r="F125" s="7"/>
     </row>
     <row r="126" spans="1:6" ht="14.25" customHeight="1">
       <c r="A126" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B126" s="1">
         <v>700813</v>
@@ -3813,14 +3813,14 @@
         <v>4005808516667</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E126" s="5"/>
       <c r="F126" s="7"/>
     </row>
     <row r="127" spans="1:6" ht="14.25" customHeight="1">
       <c r="A127" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B127" s="1">
         <v>702256</v>
@@ -3829,14 +3829,14 @@
         <v>4005900308719</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E127" s="5"/>
       <c r="F127" s="7"/>
     </row>
     <row r="128" spans="1:6" ht="14.25" customHeight="1">
       <c r="A128" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B128" s="1">
         <v>703425</v>
@@ -3845,14 +3845,14 @@
         <v>4005900694362</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>114</v>
+        <v>207</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="7"/>
     </row>
     <row r="129" spans="1:6" ht="14.25" customHeight="1">
       <c r="A129" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B129" s="1">
         <v>700765</v>
@@ -3861,14 +3861,14 @@
         <v>4005808555383</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>115</v>
+        <v>208</v>
       </c>
       <c r="E129" s="5"/>
       <c r="F129" s="7"/>
     </row>
     <row r="130" spans="1:6" ht="14.25" customHeight="1">
       <c r="A130" s="1" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B130" s="1">
         <v>701720</v>
@@ -3877,94 +3877,94 @@
         <v>4005808956487</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>116</v>
+        <v>209</v>
       </c>
       <c r="E130" s="5"/>
       <c r="F130" s="7"/>
     </row>
     <row r="131" spans="1:6" ht="14.25" customHeight="1">
       <c r="A131" s="1" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="B131" s="1">
-        <v>703785</v>
+        <v>703801</v>
       </c>
       <c r="C131" s="2">
-        <v>4006000172842</v>
+        <v>4006000172866</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="E131" s="5"/>
       <c r="F131" s="7"/>
     </row>
     <row r="132" spans="1:6" ht="14.25" customHeight="1">
       <c r="A132" s="1" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="B132" s="1">
-        <v>703793</v>
+        <v>703769</v>
       </c>
       <c r="C132" s="2">
-        <v>4006000172859</v>
+        <v>400600017282812</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
       <c r="E132" s="5"/>
       <c r="F132" s="7"/>
     </row>
     <row r="133" spans="1:6" ht="14.25" customHeight="1">
       <c r="A133" s="1" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="B133" s="1">
-        <v>703801</v>
+        <v>703777</v>
       </c>
       <c r="C133" s="2">
-        <v>4006000172866</v>
+        <v>400600017283512</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>164</v>
+        <v>212</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="7"/>
     </row>
     <row r="134" spans="1:6" ht="14.25" customHeight="1">
       <c r="A134" s="1" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="B134" s="1">
-        <v>703777</v>
+        <v>703785</v>
       </c>
       <c r="C134" s="2">
-        <v>400600017283512</v>
+        <v>4006000172842</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>151</v>
+        <v>210</v>
       </c>
       <c r="E134" s="5"/>
       <c r="F134" s="7"/>
     </row>
     <row r="135" spans="1:6" ht="14.25" customHeight="1">
       <c r="A135" s="1" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="B135" s="1">
-        <v>703769</v>
+        <v>703793</v>
       </c>
       <c r="C135" s="2">
-        <v>400600017282812</v>
+        <v>4006000172859</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>152</v>
+        <v>211</v>
       </c>
       <c r="E135" s="5"/>
       <c r="F135" s="7"/>
     </row>
     <row r="136" spans="1:6" ht="14.25" customHeight="1">
       <c r="A136" s="1" t="s">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="B136" s="1">
         <v>703473</v>
@@ -3973,14 +3973,14 @@
         <v>4005900945709</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E136" s="5"/>
       <c r="F136" s="7"/>
     </row>
     <row r="137" spans="1:6" ht="14.25" customHeight="1">
       <c r="A137" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B137" s="1">
         <v>703505</v>
@@ -3989,7 +3989,7 @@
         <v>4005808189625</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>5</v>
@@ -3998,7 +3998,7 @@
     </row>
     <row r="138" spans="1:6" ht="14.25" customHeight="1">
       <c r="A138" s="1" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="B138" s="1">
         <v>703105</v>
@@ -4007,14 +4007,14 @@
         <v>4005900602220</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="7"/>
     </row>
     <row r="139" spans="1:6" ht="14.25" customHeight="1">
       <c r="A139" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B139" s="1">
         <v>703617</v>
@@ -4023,14 +4023,14 @@
         <v>4005808189342</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="7"/>
     </row>
     <row r="140" spans="1:6" ht="14.25" customHeight="1">
       <c r="A140" s="1" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="B140" s="1">
         <v>702793</v>
@@ -4039,7 +4039,7 @@
         <v>4005900734082</v>
       </c>
       <c r="D140" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>5</v>
@@ -4048,7 +4048,7 @@
     </row>
     <row r="141" spans="1:6" ht="14.25" customHeight="1">
       <c r="A141" s="1" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="B141" s="1">
         <v>701856</v>
@@ -4057,7 +4057,7 @@
         <v>4005900095268</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="E141" s="5" t="s">
         <v>5</v>
@@ -4066,7 +4066,7 @@
     </row>
     <row r="142" spans="1:6" ht="14.25" customHeight="1">
       <c r="A142" s="1" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="B142" s="1">
         <v>702777</v>
@@ -4075,14 +4075,14 @@
         <v>4005900734068</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="E142" s="5"/>
       <c r="F142" s="7"/>
     </row>
     <row r="143" spans="1:6" ht="14.25" customHeight="1">
       <c r="A143" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B143" s="1">
         <v>700653</v>
@@ -4091,14 +4091,14 @@
         <v>4005808513550</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="E143" s="5"/>
       <c r="F143" s="7"/>
     </row>
     <row r="144" spans="1:6" ht="14.25" customHeight="1">
       <c r="A144" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B144" s="1">
         <v>703809</v>
@@ -4107,14 +4107,14 @@
         <v>4005805514260</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="E144" s="5"/>
       <c r="F144" s="7"/>
     </row>
     <row r="145" spans="1:6" ht="14.25" customHeight="1">
       <c r="A145" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B145" s="1">
         <v>703913</v>
@@ -4123,14 +4123,14 @@
         <v>4006000170237</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>166</v>
+        <v>150</v>
       </c>
       <c r="E145" s="5"/>
       <c r="F145" s="7"/>
     </row>
     <row r="146" spans="1:6" ht="14.25" customHeight="1">
       <c r="A146" s="1" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="B146" s="1">
         <v>702785</v>
@@ -4139,7 +4139,7 @@
         <v>4005900734075</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>5</v>
@@ -4148,7 +4148,7 @@
     </row>
     <row r="147" spans="1:6" ht="14.25" customHeight="1">
       <c r="A147" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B147" s="1">
         <v>700685</v>
@@ -4157,14 +4157,14 @@
         <v>7890704810738</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E147" s="5"/>
       <c r="F147" s="7"/>
     </row>
     <row r="148" spans="1:6" ht="14.25" customHeight="1">
       <c r="A148" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B148" s="1">
         <v>700645</v>
@@ -4173,14 +4173,14 @@
         <v>4005808808243</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="E148" s="5"/>
       <c r="F148" s="7"/>
     </row>
     <row r="149" spans="1:6" ht="14.25" customHeight="1">
       <c r="A149" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B149" s="1">
         <v>702881</v>
@@ -4189,14 +4189,14 @@
         <v>4005808896134</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>128</v>
+        <v>214</v>
       </c>
       <c r="E149" s="5"/>
       <c r="F149" s="7"/>
     </row>
     <row r="150" spans="1:6" ht="14.25" customHeight="1">
       <c r="A150" s="1" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B150" s="1">
         <v>702921</v>
@@ -4205,14 +4205,14 @@
         <v>4005900219626</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="E150" s="5"/>
       <c r="F150" s="7"/>
     </row>
     <row r="151" spans="1:6" ht="14.25" customHeight="1">
       <c r="A151" s="1" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B151" s="1">
         <v>701928</v>
@@ -4221,14 +4221,14 @@
         <v>7890704808131</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E151" s="5"/>
       <c r="F151" s="7"/>
     </row>
     <row r="152" spans="1:6" ht="14.25" customHeight="1">
       <c r="A152" s="1" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B152" s="1">
         <v>700701</v>
@@ -4237,7 +4237,7 @@
         <v>7890704810516</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E152" s="5" t="s">
         <v>5</v>
@@ -4246,7 +4246,7 @@
     </row>
     <row r="153" spans="1:6" ht="14.25" customHeight="1">
       <c r="A153" s="1" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B153" s="1">
         <v>703945</v>
@@ -4255,14 +4255,14 @@
         <v>4005900964380</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="E153" s="5"/>
       <c r="F153" s="7"/>
     </row>
     <row r="154" spans="1:6" ht="14.25" customHeight="1">
       <c r="A154" s="1" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B154" s="1">
         <v>700661</v>
@@ -4271,14 +4271,14 @@
         <v>4005808808281</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="E154" s="5"/>
       <c r="F154" s="7"/>
     </row>
     <row r="155" spans="1:6" ht="14.25" customHeight="1">
       <c r="A155" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B155" s="1">
         <v>702873</v>
@@ -4287,14 +4287,14 @@
         <v>4005808313167</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>133</v>
+        <v>215</v>
       </c>
       <c r="E155" s="5"/>
       <c r="F155" s="7"/>
     </row>
     <row r="156" spans="1:6" ht="14.25" customHeight="1">
       <c r="A156" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B156" s="1">
         <v>703065</v>
@@ -4303,14 +4303,14 @@
         <v>4005900916129</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="E156" s="5"/>
       <c r="F156" s="7"/>
     </row>
     <row r="157" spans="1:6" ht="14.25" customHeight="1">
       <c r="A157" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B157" s="1">
         <v>701936</v>
@@ -4319,7 +4319,7 @@
         <v>4005900294722</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="E157" s="5" t="s">
         <v>5</v>
@@ -4328,7 +4328,7 @@
     </row>
     <row r="158" spans="1:6" ht="14.25" customHeight="1">
       <c r="A158" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B158" s="1">
         <v>703121</v>
@@ -4337,14 +4337,14 @@
         <v>4005900701367</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="E158" s="5"/>
       <c r="F158" s="7"/>
     </row>
     <row r="159" spans="1:6" ht="14.25" customHeight="1">
       <c r="A159" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B159" s="1">
         <v>702841</v>
@@ -4353,14 +4353,14 @@
         <v>4005900696847</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="E159" s="5"/>
       <c r="F159" s="7"/>
     </row>
     <row r="160" spans="1:6" ht="14.25" customHeight="1">
       <c r="A160" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B160" s="1">
         <v>702448</v>
@@ -4369,14 +4369,14 @@
         <v>4005900521897</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="E160" s="5"/>
       <c r="F160" s="7"/>
     </row>
     <row r="161" spans="1:6" ht="14.25" customHeight="1">
       <c r="A161" s="1" t="s">
-        <v>207</v>
+        <v>189</v>
       </c>
       <c r="B161" s="1">
         <v>702809</v>
@@ -4385,14 +4385,14 @@
         <v>4005900742414</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="E161" s="5"/>
       <c r="F161" s="7"/>
     </row>
     <row r="162" spans="1:6" ht="14.25" customHeight="1">
       <c r="A162" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B162" s="1">
         <v>702416</v>
@@ -4401,7 +4401,7 @@
         <v>4005900521934</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="E162" s="5" t="s">
         <v>5</v>
@@ -4410,7 +4410,7 @@
     </row>
     <row r="163" spans="1:6" ht="14.25" customHeight="1">
       <c r="A163" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B163" s="1">
         <v>702825</v>
@@ -4419,14 +4419,14 @@
         <v>4005900696823</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="E163" s="5"/>
       <c r="F163" s="7"/>
     </row>
     <row r="164" spans="1:6" ht="14.25" customHeight="1">
       <c r="A164" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B164" s="1">
         <v>702400</v>
@@ -4435,14 +4435,14 @@
         <v>4005900521972</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="E164" s="5"/>
       <c r="F164" s="7"/>
     </row>
     <row r="165" spans="1:6" ht="14.25" customHeight="1">
       <c r="A165" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B165" s="1">
         <v>702464</v>
@@ -4451,14 +4451,14 @@
         <v>4005900522016</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="E165" s="5"/>
       <c r="F165" s="7"/>
     </row>
     <row r="166" spans="1:6" ht="14.25" customHeight="1">
       <c r="A166" s="1" t="s">
-        <v>207</v>
+        <v>189</v>
       </c>
       <c r="B166" s="1">
         <v>702801</v>
@@ -4467,14 +4467,14 @@
         <v>4005900742407</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="E166" s="5"/>
       <c r="F166" s="7"/>
     </row>
     <row r="167" spans="1:6" ht="14.25" customHeight="1">
       <c r="A167" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B167" s="1">
         <v>702472</v>
@@ -4483,16 +4483,16 @@
         <v>4005900521910</v>
       </c>
       <c r="D167" s="1" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="E167" s="5" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="F167" s="7"/>
     </row>
     <row r="168" spans="1:6" ht="14.25" customHeight="1">
       <c r="A168" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B168" s="1">
         <v>702761</v>
@@ -4501,14 +4501,14 @@
         <v>4005900713612</v>
       </c>
       <c r="D168" s="1" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E168" s="5"/>
       <c r="F168" s="7"/>
     </row>
     <row r="169" spans="1:6" ht="14.25" customHeight="1">
       <c r="A169" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B169" s="1">
         <v>703041</v>
@@ -4517,14 +4517,14 @@
         <v>4005900807861</v>
       </c>
       <c r="D169" s="1" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="E169" s="5"/>
       <c r="F169" s="7"/>
     </row>
     <row r="170" spans="1:6" ht="14.25" customHeight="1">
       <c r="A170" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B170" s="1">
         <v>703113</v>
@@ -4533,14 +4533,14 @@
         <v>4005900810885</v>
       </c>
       <c r="D170" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="E170" s="5"/>
       <c r="F170" s="7"/>
     </row>
     <row r="171" spans="1:6" ht="14.25" customHeight="1">
       <c r="A171" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B171" s="1">
         <v>703033</v>
@@ -4549,14 +4549,14 @@
         <v>4005900807854</v>
       </c>
       <c r="D171" s="1" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="E171" s="5"/>
       <c r="F171" s="7"/>
     </row>
     <row r="172" spans="1:6" ht="14.25" customHeight="1">
       <c r="A172" s="1" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B172" s="1">
         <v>702656</v>
@@ -4565,14 +4565,14 @@
         <v>4005900527073</v>
       </c>
       <c r="D172" s="1" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E172" s="5"/>
       <c r="F172" s="7"/>
     </row>
     <row r="173" spans="1:6" ht="14.25" customHeight="1">
       <c r="A173" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B173" s="1">
         <v>702352</v>
@@ -4581,14 +4581,14 @@
         <v>4005900380982</v>
       </c>
       <c r="D173" s="1" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="E173" s="5"/>
       <c r="F173" s="7"/>
     </row>
     <row r="174" spans="1:6" ht="14.25" customHeight="1">
       <c r="A174" s="1" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B174" s="1">
         <v>702360</v>
@@ -4597,14 +4597,14 @@
         <v>4005900380975</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
       <c r="E174" s="5"/>
       <c r="F174" s="7"/>
     </row>
     <row r="175" spans="1:6" ht="14.25" customHeight="1">
       <c r="A175" s="1" t="s">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="B175" s="1">
         <v>703097</v>
@@ -4613,7 +4613,7 @@
         <v>4005900889737</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="E175" s="5"/>
       <c r="F175" s="7"/>

</xml_diff>